<commit_message>
chore: update daily market scan
</commit_message>
<xml_diff>
--- a/output/minervini_4h.xlsx
+++ b/output/minervini_4h.xlsx
@@ -8660,10 +8660,10 @@
         <v>1988.900024414062</v>
       </c>
       <c r="I107" t="n">
-        <v>1266.16157090969</v>
+        <v>1266.161452106784</v>
       </c>
       <c r="J107" t="n">
-        <v>52.51607851267466</v>
+        <v>52.51609282313503</v>
       </c>
       <c r="K107" t="n">
         <v>2.993115300029303</v>
@@ -10662,10 +10662,10 @@
         <v>443.3731066930094</v>
       </c>
       <c r="I133" t="n">
-        <v>175.4686165435595</v>
+        <v>175.4686316122085</v>
       </c>
       <c r="J133" t="n">
-        <v>125.0829920397681</v>
+        <v>125.0829727104066</v>
       </c>
       <c r="K133" t="n">
         <v>12.26056285335546</v>
@@ -11355,10 +11355,10 @@
         <v>12865.82946046676</v>
       </c>
       <c r="I142" t="n">
-        <v>6312.244104023675</v>
+        <v>6312.244579991518</v>
       </c>
       <c r="J142" t="n">
-        <v>81.1717007697823</v>
+        <v>81.17168710873</v>
       </c>
       <c r="K142" t="n">
         <v>12.50288090649489</v>
@@ -12048,10 +12048,10 @@
         <v>394.5</v>
       </c>
       <c r="I151" t="n">
-        <v>241.7427848010177</v>
+        <v>241.7427995975111</v>
       </c>
       <c r="J151" t="n">
-        <v>58.01919396040307</v>
+        <v>58.01918428842959</v>
       </c>
       <c r="K151" t="n">
         <v>3.27225130890052</v>
@@ -16049,7 +16049,7 @@
         <v>3.87589463306528</v>
       </c>
       <c r="H203" t="n">
-        <v>2269.472002658311</v>
+        <v>2269.472253037084</v>
       </c>
       <c r="I203" t="n">
         <v>1353.205955540699</v>
@@ -16058,7 +16058,7 @@
         <v>46.68129535544045</v>
       </c>
       <c r="K203" t="n">
-        <v>14.33684189349806</v>
+        <v>14.33685450767357</v>
       </c>
       <c r="L203" t="n">
         <v>60.91794158553546</v>
@@ -25061,10 +25061,10 @@
         <v>531</v>
       </c>
       <c r="I320" t="n">
-        <v>374.3676224032645</v>
+        <v>374.3675923313683</v>
       </c>
       <c r="J320" t="n">
-        <v>28.97750158089127</v>
+        <v>28.97751194129139</v>
       </c>
       <c r="K320" t="n">
         <v>9.972039616410754</v>
@@ -26213,7 +26213,7 @@
         <v>1.72549589427522</v>
       </c>
       <c r="H335" t="n">
-        <v>3039.742428602358</v>
+        <v>3039.742679715149</v>
       </c>
       <c r="I335" t="n">
         <v>2053.692522278021</v>
@@ -26222,7 +26222,7 @@
         <v>24.41005517057211</v>
       </c>
       <c r="K335" t="n">
-        <v>18.97230640322343</v>
+        <v>18.97231623151267</v>
       </c>
       <c r="L335" t="n">
         <v>47.8442280945758</v>
@@ -26444,7 +26444,7 @@
         <v>5.337363461032152</v>
       </c>
       <c r="H338" t="n">
-        <v>297.5473847088064</v>
+        <v>297.5474157032224</v>
       </c>
       <c r="I338" t="n">
         <v>165</v>
@@ -26453,7 +26453,7 @@
         <v>41.13333037405302</v>
       </c>
       <c r="K338" t="n">
-        <v>27.77403312911619</v>
+        <v>27.77404643886696</v>
       </c>
       <c r="L338" t="n">
         <v>46.87065368567455</v>
@@ -27137,7 +27137,7 @@
         <v>3.172218883389966</v>
       </c>
       <c r="H347" t="n">
-        <v>1304.859850069017</v>
+        <v>1304.859727076846</v>
       </c>
       <c r="I347" t="n">
         <v>734.1152411860135</v>
@@ -27146,7 +27146,7 @@
         <v>39.85541963591042</v>
       </c>
       <c r="K347" t="n">
-        <v>27.09261830388225</v>
+        <v>27.09260632451378</v>
       </c>
       <c r="L347" t="n">
         <v>41.1682892906815</v>
@@ -27214,7 +27214,7 @@
         <v>1.075268063604451</v>
       </c>
       <c r="H348" t="n">
-        <v>533.7088183031568</v>
+        <v>533.7087547028075</v>
       </c>
       <c r="I348" t="n">
         <v>363.2227809620478</v>
@@ -27223,7 +27223,7 @@
         <v>21.97747801486656</v>
       </c>
       <c r="K348" t="n">
-        <v>20.46243832706111</v>
+        <v>20.46242397194295</v>
       </c>
       <c r="L348" t="n">
         <v>40.89012517385257</v>
@@ -31837,10 +31837,10 @@
         <v>1093.53919041171</v>
       </c>
       <c r="I408" t="n">
-        <v>491.2850813456647</v>
+        <v>491.2850236715819</v>
       </c>
       <c r="J408" t="n">
-        <v>47.00222734809576</v>
+        <v>47.00224460532571</v>
       </c>
       <c r="K408" t="n">
         <v>51.41777512158614</v>
@@ -35376,7 +35376,7 @@
         <v>-1.290586178552477</v>
       </c>
       <c r="H454" t="n">
-        <v>1766.733188761222</v>
+        <v>1766.733060850261</v>
       </c>
       <c r="I454" t="n">
         <v>894.2209017899434</v>
@@ -35385,7 +35385,7 @@
         <v>49.80638149974889</v>
       </c>
       <c r="K454" t="n">
-        <v>31.88513145414607</v>
+        <v>31.88512190570145</v>
       </c>
       <c r="L454" t="n">
         <v>73.57440890125174</v>
@@ -38995,7 +38995,7 @@
         <v>-0.5888225702531225</v>
       </c>
       <c r="H501" t="n">
-        <v>3287.161645949698</v>
+        <v>3287.161392369851</v>
       </c>
       <c r="I501" t="n">
         <v>1966.020518717901</v>
@@ -39004,7 +39004,7 @@
         <v>19.12388389147057</v>
       </c>
       <c r="K501" t="n">
-        <v>40.35703014302723</v>
+        <v>40.35701931553588</v>
       </c>
       <c r="L501" t="n">
         <v>19.05424200278164</v>
@@ -39383,10 +39383,10 @@
         <v>872.0425606177564</v>
       </c>
       <c r="I506" t="n">
-        <v>406.1171468902937</v>
+        <v>406.117116732523</v>
       </c>
       <c r="J506" t="n">
-        <v>25.44410303972004</v>
+        <v>25.44411235504889</v>
       </c>
       <c r="K506" t="n">
         <v>71.17333197027662</v>
@@ -39691,10 +39691,10 @@
         <v>387.7999877929688</v>
       </c>
       <c r="I510" t="n">
-        <v>217.6006723249054</v>
+        <v>217.6006872017223</v>
       </c>
       <c r="J510" t="n">
-        <v>24.08049897789644</v>
+        <v>24.08049049482182</v>
       </c>
       <c r="K510" t="n">
         <v>43.62962510850694</v>
@@ -40535,7 +40535,7 @@
         <v>0.1647393729975022</v>
       </c>
       <c r="H521" t="n">
-        <v>87.39771312453149</v>
+        <v>87.39772087555167</v>
       </c>
       <c r="I521" t="n">
         <v>71.42454681386315</v>
@@ -40544,7 +40544,7 @@
         <v>4.753901890074053</v>
       </c>
       <c r="K521" t="n">
-        <v>16.81063015371458</v>
+        <v>16.81064051327112</v>
       </c>
       <c r="L521" t="n">
         <v>39.91655076495132</v>
@@ -41305,7 +41305,7 @@
         <v>0.5286217519214098</v>
       </c>
       <c r="H531" t="n">
-        <v>155.8999606999571</v>
+        <v>155.8999783750524</v>
       </c>
       <c r="I531" t="n">
         <v>112.8155071321618</v>
@@ -41314,7 +41314,7 @@
         <v>7.963883820573336</v>
       </c>
       <c r="K531" t="n">
-        <v>27.99668045468675</v>
+        <v>27.99669496625883</v>
       </c>
       <c r="L531" t="n">
         <v>31.43254520166898</v>
@@ -41613,7 +41613,7 @@
         <v>2.185911334104285</v>
       </c>
       <c r="H535" t="n">
-        <v>46547.9774954976</v>
+        <v>46547.97355089381</v>
       </c>
       <c r="I535" t="n">
         <v>29525.27549507192</v>
@@ -41622,7 +41622,7 @@
         <v>21.87862567448789</v>
       </c>
       <c r="K535" t="n">
-        <v>29.35383491870947</v>
+        <v>29.35382395690929</v>
       </c>
       <c r="L535" t="n">
         <v>28.37273991655077</v>
@@ -42460,7 +42460,7 @@
         <v>1.213630845153424</v>
       </c>
       <c r="H546" t="n">
-        <v>124.8273017901132</v>
+        <v>124.8273096544699</v>
       </c>
       <c r="I546" t="n">
         <v>76.65010804466255</v>
@@ -42469,7 +42469,7 @@
         <v>14.15509023029091</v>
       </c>
       <c r="K546" t="n">
-        <v>42.65977347441505</v>
+        <v>42.65978246225137</v>
       </c>
       <c r="L546" t="n">
         <v>20.86230876216968</v>
@@ -44773,10 +44773,10 @@
         <v>484.7737901614043</v>
       </c>
       <c r="I576" t="n">
-        <v>349.5720248388532</v>
+        <v>349.5720548957738</v>
       </c>
       <c r="J576" t="n">
-        <v>14.71169644792205</v>
+        <v>14.71168658477568</v>
       </c>
       <c r="K576" t="n">
         <v>20.89121949162202</v>
@@ -45925,7 +45925,7 @@
         <v>1.553058150552844</v>
       </c>
       <c r="H591" t="n">
-        <v>239.2186728978909</v>
+        <v>239.2186883393384</v>
       </c>
       <c r="I591" t="n">
         <v>156.7443123050878</v>
@@ -45934,7 +45934,7 @@
         <v>16.68684573414505</v>
       </c>
       <c r="K591" t="n">
-        <v>30.7920617172252</v>
+        <v>30.79207015978833</v>
       </c>
       <c r="L591" t="n">
         <v>26.56467315716273</v>
@@ -46926,7 +46926,7 @@
         <v>-0.446131700275032</v>
       </c>
       <c r="H604" t="n">
-        <v>294.6532203195111</v>
+        <v>294.6532543042141</v>
       </c>
       <c r="I604" t="n">
         <v>213.7350670269712</v>
@@ -46935,7 +46935,7 @@
         <v>5.803882598783772</v>
       </c>
       <c r="K604" t="n">
-        <v>30.29681662455992</v>
+        <v>30.29683165272965</v>
       </c>
       <c r="L604" t="n">
         <v>20.72322670375522</v>
@@ -47234,7 +47234,7 @@
         <v>0.7510223845656139</v>
       </c>
       <c r="H608" t="n">
-        <v>408.554305468849</v>
+        <v>408.5542740377988</v>
       </c>
       <c r="I608" t="n">
         <v>243.9284560598348</v>
@@ -47243,7 +47243,7 @@
         <v>14.33680120865899</v>
       </c>
       <c r="K608" t="n">
-        <v>46.48774270697429</v>
+        <v>46.48773143732537</v>
       </c>
       <c r="L608" t="n">
         <v>17.94158553546593</v>
@@ -47388,7 +47388,7 @@
         <v>0.1706315473898767</v>
       </c>
       <c r="H610" t="n">
-        <v>2448.345231432346</v>
+        <v>2448.345479475883</v>
       </c>
       <c r="I610" t="n">
         <v>1761.237851420491</v>
@@ -47397,7 +47397,7 @@
         <v>3.728183160531828</v>
       </c>
       <c r="K610" t="n">
-        <v>34.01637739961159</v>
+        <v>34.01639097690283</v>
       </c>
       <c r="L610" t="n">
         <v>16.82892906815021</v>
@@ -48774,7 +48774,7 @@
         <v>0.6477673935719519</v>
       </c>
       <c r="H628" t="n">
-        <v>372.3009385265751</v>
+        <v>372.3009694554414</v>
       </c>
       <c r="I628" t="n">
         <v>218.8999938964844</v>
@@ -48783,7 +48783,7 @@
         <v>9.365007113565404</v>
       </c>
       <c r="K628" t="n">
-        <v>55.5141804588168</v>
+        <v>55.51419337814305</v>
       </c>
       <c r="L628" t="n">
         <v>5.285118219749652</v>
@@ -52624,7 +52624,7 @@
         <v>-1.006731507353509</v>
       </c>
       <c r="H678" t="n">
-        <v>263.220498300555</v>
+        <v>263.2205288662585</v>
       </c>
       <c r="I678" t="n">
         <v>167.0916913788894</v>
@@ -52633,7 +52633,7 @@
         <v>8.293832838120196</v>
       </c>
       <c r="K678" t="n">
-        <v>45.46587606511259</v>
+        <v>45.46589295690811</v>
       </c>
       <c r="L678" t="n">
         <v>11.82197496522948</v>
@@ -52932,7 +52932,7 @@
         <v>-0.4425166749201459</v>
       </c>
       <c r="H682" t="n">
-        <v>97.9287679734358</v>
+        <v>97.92876001560526</v>
       </c>
       <c r="I682" t="n">
         <v>62.68610889438828</v>
@@ -52941,7 +52941,7 @@
         <v>3.627422773864231</v>
       </c>
       <c r="K682" t="n">
-        <v>50.75241587687098</v>
+        <v>50.75240362651592</v>
       </c>
       <c r="L682" t="n">
         <v>10.84840055632823</v>
@@ -53086,7 +53086,7 @@
         <v>-1.193779559056574</v>
       </c>
       <c r="H684" t="n">
-        <v>1284.135475005729</v>
+        <v>1284.135346691241</v>
       </c>
       <c r="I684" t="n">
         <v>902.8120757721283</v>
@@ -53095,7 +53095,7 @@
         <v>1.349995702865181</v>
       </c>
       <c r="K684" t="n">
-        <v>40.34267486401415</v>
+        <v>40.34266084057276</v>
       </c>
       <c r="L684" t="n">
         <v>10.43115438108484</v>
@@ -55396,7 +55396,7 @@
         <v>-1.971118231218572</v>
       </c>
       <c r="H714" t="n">
-        <v>1343.927192495164</v>
+        <v>1343.927068287785</v>
       </c>
       <c r="I714" t="n">
         <v>680.1500244140625</v>
@@ -55405,7 +55405,7 @@
         <v>4.035867115570957</v>
       </c>
       <c r="K714" t="n">
-        <v>89.92753517017964</v>
+        <v>89.92751761684681</v>
       </c>
       <c r="L714" t="n">
         <v>1.390820584144645</v>

</xml_diff>